<commit_message>
RFP-027 Rev 02: final terminology pass (SAMA Submitted Programme / Assessed)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULHmTMMSFeFXCeQAWPh5ca
</commit_message>
<xml_diff>
--- a/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
+++ b/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
@@ -326,7 +326,7 @@
     <t xml:space="preserve">ASSESSED RATE BUILD-UPS</t>
   </si>
   <si>
-    <t xml:space="preserve">How to read this tab: each line is quantity x rate = amount, with the reason beside it ('Basis': what the line buys, how many, how long, the rate and where the quantity comes from). Item totals go to column J of the 'Assessment' tab; the 'Return' link on each total row goes back there. A quantity in blue is a link to the 'Programme' tab row it is calculated from - click it. Units: a 'month' is 30.4 calendar days; a 'day' is one calendar day of hire or attendance; a 'man-day' is one person for one working day; working days exclude Fridays. 'Needs confirmation' marks an assessment allowance the Contractor has not yet substantiated; 'Provisional' marks a scope or price awaiting a document. All amounts exclude VAT.</t>
+    <t xml:space="preserve">How to read this tab: each line is quantity x rate = amount, with the reason beside it ('Basis': what the line buys, how many, how long, the rate and where the quantity comes from). Item totals go to column J of the 'Assessment' tab; the 'Return' link on each total row goes back there. A quantity in blue is a link to the 'Programme' tab row it is calculated from - click it. Units: a 'month' is 30.4 calendar days; a 'day' is one calendar day of hire or attendance; a 'man-day' is one person for one working day; working days exclude Fridays. 'Needs confirmation' marks an assessed allowance the Contractor has not yet substantiated; 'Provisional' marks a scope or price awaiting a document. All amounts exclude VAT.</t>
   </si>
   <si>
     <t xml:space="preserve">Back to 'Assessment'</t>
@@ -2351,7 +2351,7 @@
     <t xml:space="preserve">-</t>
   </si>
   <si>
-    <t xml:space="preserve">Activity QCD18TSECONIF2050, 03-Dec-2026, zero duration. An interface milestone outside the Contractor's control, taken as submitted in the submitted programme and in the assessment allowance; it, not the tank erection, fixes the earliest tie-in date</t>
+    <t xml:space="preserve">Activity QCD18TSECONIF2050, 03-Dec-2026, zero duration. An interface milestone outside the Contractor's control, taken as submitted in the SAMA Submitted Programme and in the Assessed basis; it, not the tank erection, fixes the earliest tie-in date</t>
   </si>
   <si>
     <t xml:space="preserve">P16</t>
@@ -2471,7 +2471,7 @@
     <t xml:space="preserve">Erection window - Tank 1 base panels start to Tank 2 mechanical finish (calendar days)</t>
   </si>
   <si>
-    <t xml:space="preserve">Power tools and lighting towers are hired by the month while erection is in progress, 12-Sep to 03-Dec-2026 as submitted; the same in the submitted programme and in the assessment allowance</t>
+    <t xml:space="preserve">Power tools and lighting towers are hired by the month while erection is in progress, 12-Sep to 03-Dec-2026 as submitted; the same in the SAMA Submitted Programme and in the Assessed basis</t>
   </si>
   <si>
     <t xml:space="preserve">D6</t>
@@ -3413,7 +3413,7 @@
     <t xml:space="preserve">Transfer hoses: not needed as submitted; 1 week allowed</t>
   </si>
   <si>
-    <t xml:space="preserve">Nil in the submitted programme and in the assessment allowance: the transfer labour is within the approved histogram helpers priced at 5.10 (Section 4, week W16)</t>
+    <t xml:space="preserve">Nil in the SAMA Submitted Programme and in the Assessed basis: the transfer labour is within the approved histogram helpers priced at 5.10 (Section 4, week W16)</t>
   </si>
   <si>
     <t xml:space="preserve">Top-up at 10 per cent of the water filled: of two fills on the SAMA Submitted Programme, of one fill in the Assessed basis (retention in Tank 1 between P18 and P19)</t>

</xml_diff>

<commit_message>
RFP-027 Rev 02: Assessment print one page wide; 2.1 and 2.5 wording; follow-up request placeholder removed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULHmTMMSFeFXCeQAWPh5ca
</commit_message>
<xml_diff>
--- a/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
+++ b/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
@@ -621,7 +621,7 @@
     <t xml:space="preserve">2.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Design engineer - coordination, review of supplier calculations, method statements, ITPs</t>
+    <t xml:space="preserve">Design engineer - design coordination and review of the supplier's calculations, method statements and ITPs</t>
   </si>
   <si>
     <t xml:space="preserve">• 2 months retained: the programme shows shop drawings 07 to 25-Aug-2026 (activities QCD18TSEENG1240 and 1250) with resubmissions to 29-Sep-2026 and the pipework shop drawings still in preparation, consistent with the period assessed
@@ -673,7 +673,8 @@
     <t xml:space="preserve">• Quantity: 12.5 engineer-days for the nine documents the programme requires for this works package (QCD18TSEMOB1050 and 1080 to 1150): tank installation (with the supplier's input), pipe installation and tie-in method statements at 2 days each; HSE, CEMP, quality, execution and mobilisation plans at 1 day each, as extensions of the contract-level plans; the ITP at 1.5 days; each with one resubmission
 • Project documents for a separate site, not head-office overheads, so priced here and not in the Overhead and Profit ('Assessment' tab, row 20)
 • The dismantling method statement is inside the Item 3 quotation; submittal administration is 2.4
-• Rate: assessed allowance (Riyadh market, Sep-2026)</t>
+• Rate: assessed allowance (Riyadh market, Sep-2026)
+• Prepared 21-Jul to 15-Aug-2026, before the Item 1 site staff start on 22-Aug-2026; the design engineer at 2.1 reviews them, he does not write them</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL ITEM 2 - goes to 'Assessment' item 2, column J</t>
@@ -2011,7 +2012,7 @@
     <t xml:space="preserve">Revalidated supplier quotations; both had lapsed before the proposal was submitted</t>
   </si>
   <si>
-    <t xml:space="preserve">WT Partnership Aconex substantiation request dated 25-Aug-2026; WT Partnership follow-up clarification request (issue to be confirmed).</t>
+    <t xml:space="preserve">WT Partnership Aconex substantiation request dated 25-Aug-2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Not received</t>
@@ -8542,7 +8543,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.354166666666667" right="0.354166666666667" top="0.5" bottom="0.433333333333333" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -21400,7 +21401,7 @@
       </c>
       <c r="B238" s="78" t="str">
         <f aca="false">'Build-Up'!B37</f>
-        <v>Design engineer - coordination, review of supplier calculations, method statements, ITPs</v>
+        <v>Design engineer - design coordination and review of the supplier's calculations, method statements and ITPs</v>
       </c>
       <c r="C238" s="86" t="s">
         <v>1236</v>

</xml_diff>

<commit_message>
RFP-027 Rev 02 final: assumptions 2 and 4 as bullet lists
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULHmTMMSFeFXCeQAWPh5ca
</commit_message>
<xml_diff>
--- a/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
+++ b/deliverables/RFP-027/Qiddiya - TSE Irrigation Storage Tanks - Cost Assessment - Rev 02 - 30 Sep 2026.xlsx
@@ -1579,7 +1579,23 @@
 • The Daywork Schedule applies only to Engineer-instructed daywork and is not used</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Rates marked 'assessed allowance' or 'assumption' are assessed Riyadh market rates (Sep-2026): crane 50 t SAR 2,500/day; boom truck SAR 1,200/day and telehandler SAR 900/day, both with operator and fuel; scaffolding SAR 55/m2; generator 100 kVA SAR 11,000/month with fuel; general labour SAR 150/day (helpers SAR 3,900 per person-month at 26 working days); rigger SAR 250/day; site engineer SAR 12,000/month; HSE and QA/QC SAR 10,000/month; foreman SAR 8,000/month; test water SAR 15.00/m3 tankered (one 30 m3 load at the local haulage rate); site water SAR 350 per 10 m3 delivery; generator 30 kVA SAR 8,571/month continuous with fuel (hire SAR 4,000 plus diesel at SAR 1.79 a litre); local haulage SAR 450/load; HDPE PE100 pipe 355 mm outside diameter supplied and installed SAR 280/m; gate valve DN300 SAR 6,500; motorised butterfly valve DN355 as listed SAR 14,000 excluding power and control.</t>
+    <t xml:space="preserve">2. Rates marked 'assessed allowance' or 'assumption' are assessed Riyadh market rates (Sep-2026):
+• crane 50 t SAR 2,500/day
+• boom truck SAR 1,200/day and telehandler SAR 900/day, both with operator and fuel
+• scaffolding SAR 55/m2
+• generator 100 kVA SAR 11,000/month with fuel
+• general labour SAR 150/day (helpers SAR 3,900 per person-month at 26 working days)
+• rigger SAR 250/day
+• site engineer SAR 12,000/month
+• HSE and QA/QC SAR 10,000/month
+• foreman SAR 8,000/month
+• test water SAR 15.00/m3 tankered (one 30 m3 load at the local haulage rate)
+• site water SAR 350 per 10 m3 delivery
+• generator 30 kVA SAR 8,571/month continuous with fuel (hire SAR 4,000 plus diesel at SAR 1.79 a litre)
+• local haulage SAR 450/load
+• HDPE PE100 pipe 355 mm outside diameter supplied and installed SAR 280/m
+• gate valve DN300 SAR 6,500
+• motorised butterfly valve DN355 as listed SAR 14,000 excluding power and control</t>
   </si>
   <si>
     <t xml:space="preserve">3. Programme: every period on this tab comes from the Contractor's programme of 29-Sep-2026, imported as received on the 'XER WBS' tab and worked through on the 'Programme' tab
@@ -1589,7 +1605,13 @@
 • Dates after 28-Sep-2026 are forecasts</t>
   </si>
   <si>
-    <t xml:space="preserve">4. The Engineer's (KEO) email of 30-Aug-2026, relied on above: water and power are arranged by the Contractor pending the Employer's confirmation of local sources; one tank is filled and the water re-used for the second; dismantled materials are handed to the Employer at a location assumed to be local; thermal insulation is not required; the Contractor's methodology uses forklifts, cranes and pallet jacks; no CAD drawings exist beyond the marked-up schematic in the RFP.</t>
+    <t xml:space="preserve">4. The Engineer's (KEO) email of 30-Aug-2026, relied on above:
+• water and power are arranged by the Contractor pending the Employer's confirmation of local sources
+• one tank is filled and the water re-used for the second
+• dismantled materials are handed to the Employer at a location assumed to be local
+• thermal insulation is not required
+• the Contractor's methodology uses forklifts, cranes and pallet jacks
+• no CAD drawings exist beyond the marked-up schematic in the RFP</t>
   </si>
   <si>
     <t xml:space="preserve">5. The tank site is outside the D-18 site boundary
@@ -12452,7 +12474,7 @@
       <c r="F167" s="49"/>
       <c r="G167" s="49"/>
     </row>
-    <row r="168" customFormat="false" ht="63" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="223.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="49" t="s">
         <v>453</v>
       </c>
@@ -12474,7 +12496,7 @@
       <c r="F169" s="49"/>
       <c r="G169" s="49"/>
     </row>
-    <row r="170" customFormat="false" ht="38.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="49" t="s">
         <v>455</v>
       </c>

</xml_diff>